<commit_message>
Add weekly_off_day validator test for Leave Stage 1
</commit_message>
<xml_diff>
--- a/Leave-Payroll-Implementation-Tracker.xlsx
+++ b/Leave-Payroll-Implementation-Tracker.xlsx
@@ -1018,7 +1018,7 @@
       </c>
       <c r="F3" s="4" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="G3" s="4" t="inlineStr">
@@ -1070,7 +1070,7 @@
       </c>
       <c r="F4" s="4" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="G4" s="4" t="inlineStr">
@@ -1122,7 +1122,7 @@
       </c>
       <c r="F5" s="4" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Verified</t>
         </is>
       </c>
       <c r="G5" s="4" t="inlineStr">

</xml_diff>

<commit_message>
Add LeaveRequest unique index duplicate insert test
</commit_message>
<xml_diff>
--- a/Leave-Payroll-Implementation-Tracker.xlsx
+++ b/Leave-Payroll-Implementation-Tracker.xlsx
@@ -1190,7 +1190,7 @@
       </c>
       <c r="F7" s="4" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="G7" s="4" t="inlineStr">
@@ -1243,7 +1243,7 @@
       </c>
       <c r="G8" s="4" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="H8" s="4" t="inlineStr">
@@ -1295,7 +1295,7 @@
       </c>
       <c r="G9" s="4" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="H9" s="4" t="inlineStr">
@@ -1342,7 +1342,7 @@
       </c>
       <c r="F10" s="4" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Verified</t>
         </is>
       </c>
       <c r="G10" s="4" t="inlineStr">
@@ -1360,7 +1360,11 @@
           <t>Leave Stage 2</t>
         </is>
       </c>
-      <c r="J10" s="4" t="n"/>
+      <c r="J10" s="4" t="inlineStr">
+        <is>
+          <t>npm run test:leave-request-unique</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Add leave checkClash Beautician and blackout test
</commit_message>
<xml_diff>
--- a/Leave-Payroll-Implementation-Tracker.xlsx
+++ b/Leave-Payroll-Implementation-Tracker.xlsx
@@ -1410,7 +1410,7 @@
       </c>
       <c r="F12" s="4" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="G12" s="4" t="inlineStr">
@@ -1468,7 +1468,7 @@
       </c>
       <c r="H13" s="4" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="I13" s="4" t="inlineStr">
@@ -1510,7 +1510,7 @@
       </c>
       <c r="F14" s="4" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Verified</t>
         </is>
       </c>
       <c r="G14" s="4" t="inlineStr">
@@ -1528,7 +1528,11 @@
           <t>Leave Stage 3</t>
         </is>
       </c>
-      <c r="J14" s="4" t="n"/>
+      <c r="J14" s="4" t="inlineStr">
+        <is>
+          <t>npm run test:leave-clash</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Add calculateIsPaid weekly leave deduction test
</commit_message>
<xml_diff>
--- a/Leave-Payroll-Implementation-Tracker.xlsx
+++ b/Leave-Payroll-Implementation-Tracker.xlsx
@@ -1578,7 +1578,7 @@
       </c>
       <c r="F16" s="4" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="G16" s="4" t="inlineStr">
@@ -1635,7 +1635,7 @@
       </c>
       <c r="G17" s="4" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="H17" s="4" t="inlineStr">
@@ -1682,7 +1682,7 @@
       </c>
       <c r="F18" s="4" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Verified</t>
         </is>
       </c>
       <c r="G18" s="4" t="inlineStr">
@@ -1700,7 +1700,11 @@
           <t>Leave Stage 4</t>
         </is>
       </c>
-      <c r="J18" s="4" t="n"/>
+      <c r="J18" s="4" t="inlineStr">
+        <is>
+          <t>npm run test:leave-is-paid</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Add designation-clash leave swap test
</commit_message>
<xml_diff>
--- a/Leave-Payroll-Implementation-Tracker.xlsx
+++ b/Leave-Payroll-Implementation-Tracker.xlsx
@@ -907,7 +907,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J36"/>
+  <dimension ref="A1:L36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -980,15 +980,15 @@
           <t>STAGE 1 — WEEKLY OFF + BLACKOUT RULE</t>
         </is>
       </c>
-      <c r="B2" s="3" t="n"/>
-      <c r="C2" s="3" t="n"/>
-      <c r="D2" s="3" t="n"/>
-      <c r="E2" s="3" t="n"/>
-      <c r="F2" s="3" t="n"/>
-      <c r="G2" s="3" t="n"/>
-      <c r="H2" s="3" t="n"/>
-      <c r="I2" s="3" t="n"/>
-      <c r="J2" s="3" t="n"/>
+      <c r="B2" s="3" t="inlineStr"/>
+      <c r="C2" s="3" t="inlineStr"/>
+      <c r="D2" s="3" t="inlineStr"/>
+      <c r="E2" s="3" t="inlineStr"/>
+      <c r="F2" s="3" t="inlineStr"/>
+      <c r="G2" s="3" t="inlineStr"/>
+      <c r="H2" s="3" t="inlineStr"/>
+      <c r="I2" s="3" t="inlineStr"/>
+      <c r="J2" s="3" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="4" t="inlineStr">
@@ -1152,15 +1152,15 @@
           <t>STAGE 2 — LEAVEREQUEST MODEL</t>
         </is>
       </c>
-      <c r="B6" s="3" t="n"/>
-      <c r="C6" s="3" t="n"/>
-      <c r="D6" s="3" t="n"/>
-      <c r="E6" s="3" t="n"/>
-      <c r="F6" s="3" t="n"/>
-      <c r="G6" s="3" t="n"/>
-      <c r="H6" s="3" t="n"/>
-      <c r="I6" s="3" t="n"/>
-      <c r="J6" s="3" t="n"/>
+      <c r="B6" s="3" t="inlineStr"/>
+      <c r="C6" s="3" t="inlineStr"/>
+      <c r="D6" s="3" t="inlineStr"/>
+      <c r="E6" s="3" t="inlineStr"/>
+      <c r="F6" s="3" t="inlineStr"/>
+      <c r="G6" s="3" t="inlineStr"/>
+      <c r="H6" s="3" t="inlineStr"/>
+      <c r="I6" s="3" t="inlineStr"/>
+      <c r="J6" s="3" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
@@ -1208,7 +1208,7 @@
           <t>Leave Stage 2</t>
         </is>
       </c>
-      <c r="J7" s="4" t="n"/>
+      <c r="J7" s="4" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
@@ -1261,6 +1261,11 @@
           <t>Leave Stage 2</t>
         </is>
       </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>Declared on LeaveRequest.js — duplicate rejection verified in row 10.</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
@@ -1313,6 +1318,16 @@
           <t>Leave Stage 2</t>
         </is>
       </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>Declared on LeaveRequest.js — leaveRequestSchema.index({ date: 1</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> status: 1 }).</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
@@ -1372,15 +1387,15 @@
           <t>STAGE 3 — CLASH CHECKER</t>
         </is>
       </c>
-      <c r="B11" s="3" t="n"/>
-      <c r="C11" s="3" t="n"/>
-      <c r="D11" s="3" t="n"/>
-      <c r="E11" s="3" t="n"/>
-      <c r="F11" s="3" t="n"/>
-      <c r="G11" s="3" t="n"/>
-      <c r="H11" s="3" t="n"/>
-      <c r="I11" s="3" t="n"/>
-      <c r="J11" s="3" t="n"/>
+      <c r="B11" s="3" t="inlineStr"/>
+      <c r="C11" s="3" t="inlineStr"/>
+      <c r="D11" s="3" t="inlineStr"/>
+      <c r="E11" s="3" t="inlineStr"/>
+      <c r="F11" s="3" t="inlineStr"/>
+      <c r="G11" s="3" t="inlineStr"/>
+      <c r="H11" s="3" t="inlineStr"/>
+      <c r="I11" s="3" t="inlineStr"/>
+      <c r="J11" s="3" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="4" t="inlineStr">
@@ -1428,7 +1443,7 @@
           <t>Leave Stage 3</t>
         </is>
       </c>
-      <c r="J12" s="4" t="n"/>
+      <c r="J12" s="4" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
@@ -1481,6 +1496,16 @@
           <t>Critical</t>
         </is>
       </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>Leave Stage 3</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>excludeStaffId used only for swaps.</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="4" t="inlineStr">
@@ -1540,15 +1565,15 @@
           <t>STAGE 4 — DEDUCTION CALCULATOR</t>
         </is>
       </c>
-      <c r="B15" s="3" t="n"/>
-      <c r="C15" s="3" t="n"/>
-      <c r="D15" s="3" t="n"/>
-      <c r="E15" s="3" t="n"/>
-      <c r="F15" s="3" t="n"/>
-      <c r="G15" s="3" t="n"/>
-      <c r="H15" s="3" t="n"/>
-      <c r="I15" s="3" t="n"/>
-      <c r="J15" s="3" t="n"/>
+      <c r="B15" s="3" t="inlineStr"/>
+      <c r="C15" s="3" t="inlineStr"/>
+      <c r="D15" s="3" t="inlineStr"/>
+      <c r="E15" s="3" t="inlineStr"/>
+      <c r="F15" s="3" t="inlineStr"/>
+      <c r="G15" s="3" t="inlineStr"/>
+      <c r="H15" s="3" t="inlineStr"/>
+      <c r="I15" s="3" t="inlineStr"/>
+      <c r="J15" s="3" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="4" t="inlineStr">
@@ -1653,6 +1678,7 @@
           <t>Leave Stage 4</t>
         </is>
       </c>
+      <c r="K17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="4" t="inlineStr">
@@ -1712,15 +1738,15 @@
           <t>STAGE 5 — LEAVE SWAP</t>
         </is>
       </c>
-      <c r="B19" s="3" t="n"/>
-      <c r="C19" s="3" t="n"/>
-      <c r="D19" s="3" t="n"/>
-      <c r="E19" s="3" t="n"/>
-      <c r="F19" s="3" t="n"/>
-      <c r="G19" s="3" t="n"/>
-      <c r="H19" s="3" t="n"/>
-      <c r="I19" s="3" t="n"/>
-      <c r="J19" s="3" t="n"/>
+      <c r="B19" s="3" t="inlineStr"/>
+      <c r="C19" s="3" t="inlineStr"/>
+      <c r="D19" s="3" t="inlineStr"/>
+      <c r="E19" s="3" t="inlineStr"/>
+      <c r="F19" s="3" t="inlineStr"/>
+      <c r="G19" s="3" t="inlineStr"/>
+      <c r="H19" s="3" t="inlineStr"/>
+      <c r="I19" s="3" t="inlineStr"/>
+      <c r="J19" s="3" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="4" t="inlineStr">
@@ -1750,7 +1776,7 @@
       </c>
       <c r="F20" s="4" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="G20" s="4" t="inlineStr">
@@ -1802,7 +1828,7 @@
       </c>
       <c r="F21" s="4" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Verified</t>
         </is>
       </c>
       <c r="G21" s="4" t="inlineStr">
@@ -1820,7 +1846,11 @@
           <t>Leave Stage 5</t>
         </is>
       </c>
-      <c r="J21" s="4" t="n"/>
+      <c r="J21" s="4" t="inlineStr">
+        <is>
+          <t>npm run test:leave-swap</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="4" t="inlineStr">
@@ -1850,7 +1880,7 @@
       </c>
       <c r="F22" s="4" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Verified</t>
         </is>
       </c>
       <c r="G22" s="4" t="inlineStr">
@@ -1868,7 +1898,11 @@
           <t>Leave Stage 5</t>
         </is>
       </c>
-      <c r="J22" s="4" t="n"/>
+      <c r="J22" s="4" t="inlineStr">
+        <is>
+          <t>npm run test:leave-swap-blackout</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="4" t="inlineStr">
@@ -1898,7 +1932,7 @@
       </c>
       <c r="F23" s="4" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Verified</t>
         </is>
       </c>
       <c r="G23" s="4" t="inlineStr">
@@ -1916,7 +1950,11 @@
           <t>Leave Stage 5</t>
         </is>
       </c>
-      <c r="J23" s="4" t="n"/>
+      <c r="J23" s="4" t="inlineStr">
+        <is>
+          <t>npm run test:leave-swap-clash</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -1924,15 +1962,15 @@
           <t>STAGE 6 — ATTENDANCE SYNC</t>
         </is>
       </c>
-      <c r="B24" s="3" t="n"/>
-      <c r="C24" s="3" t="n"/>
-      <c r="D24" s="3" t="n"/>
-      <c r="E24" s="3" t="n"/>
-      <c r="F24" s="3" t="n"/>
-      <c r="G24" s="3" t="n"/>
-      <c r="H24" s="3" t="n"/>
-      <c r="I24" s="3" t="n"/>
-      <c r="J24" s="3" t="n"/>
+      <c r="B24" s="3" t="inlineStr"/>
+      <c r="C24" s="3" t="inlineStr"/>
+      <c r="D24" s="3" t="inlineStr"/>
+      <c r="E24" s="3" t="inlineStr"/>
+      <c r="F24" s="3" t="inlineStr"/>
+      <c r="G24" s="3" t="inlineStr"/>
+      <c r="H24" s="3" t="inlineStr"/>
+      <c r="I24" s="3" t="inlineStr"/>
+      <c r="J24" s="3" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" s="4" t="inlineStr">
@@ -2084,7 +2122,7 @@
           <t>Leave Stage 6</t>
         </is>
       </c>
-      <c r="J27" s="4" t="n"/>
+      <c r="J27" s="4" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -2092,15 +2130,15 @@
           <t>STAGE 7 — LEAVE API ROUTES</t>
         </is>
       </c>
-      <c r="B28" s="3" t="n"/>
-      <c r="C28" s="3" t="n"/>
-      <c r="D28" s="3" t="n"/>
-      <c r="E28" s="3" t="n"/>
-      <c r="F28" s="3" t="n"/>
-      <c r="G28" s="3" t="n"/>
-      <c r="H28" s="3" t="n"/>
-      <c r="I28" s="3" t="n"/>
-      <c r="J28" s="3" t="n"/>
+      <c r="B28" s="3" t="inlineStr"/>
+      <c r="C28" s="3" t="inlineStr"/>
+      <c r="D28" s="3" t="inlineStr"/>
+      <c r="E28" s="3" t="inlineStr"/>
+      <c r="F28" s="3" t="inlineStr"/>
+      <c r="G28" s="3" t="inlineStr"/>
+      <c r="H28" s="3" t="inlineStr"/>
+      <c r="I28" s="3" t="inlineStr"/>
+      <c r="J28" s="3" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" s="4" t="inlineStr">
@@ -2148,7 +2186,7 @@
           <t>Leave Stage 7</t>
         </is>
       </c>
-      <c r="J29" s="4" t="n"/>
+      <c r="J29" s="4" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" s="4" t="inlineStr">
@@ -2196,7 +2234,7 @@
           <t>Leave Stage 7</t>
         </is>
       </c>
-      <c r="J30" s="4" t="n"/>
+      <c r="J30" s="4" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" s="4" t="inlineStr">
@@ -2244,7 +2282,7 @@
           <t>Leave Stage 7</t>
         </is>
       </c>
-      <c r="J31" s="4" t="n"/>
+      <c r="J31" s="4" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" s="4" t="inlineStr">
@@ -2292,7 +2330,7 @@
           <t>Leave Stage 7</t>
         </is>
       </c>
-      <c r="J32" s="4" t="n"/>
+      <c r="J32" s="4" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" s="4" t="inlineStr">
@@ -2340,7 +2378,7 @@
           <t>Leave Stage 7</t>
         </is>
       </c>
-      <c r="J33" s="4" t="n"/>
+      <c r="J33" s="4" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" s="4" t="inlineStr">
@@ -2388,7 +2426,7 @@
           <t>Leave Stage 7</t>
         </is>
       </c>
-      <c r="J34" s="4" t="n"/>
+      <c r="J34" s="4" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" s="4" t="inlineStr">
@@ -2436,7 +2474,7 @@
           <t>Leave Stage 7</t>
         </is>
       </c>
-      <c r="J35" s="4" t="n"/>
+      <c r="J35" s="4" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" s="4" t="inlineStr">
@@ -2484,7 +2522,7 @@
           <t>Leave Stage 7</t>
         </is>
       </c>
-      <c r="J36" s="4" t="n"/>
+      <c r="J36" s="4" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Add syncAttendanceForLeave to upsert on_leave attendance
</commit_message>
<xml_diff>
--- a/Leave-Payroll-Implementation-Tracker.xlsx
+++ b/Leave-Payroll-Implementation-Tracker.xlsx
@@ -2000,7 +2000,7 @@
       </c>
       <c r="F25" s="4" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Verified</t>
         </is>
       </c>
       <c r="G25" s="4" t="inlineStr">
@@ -2020,7 +2020,7 @@
       </c>
       <c r="J25" s="4" t="inlineStr">
         <is>
-          <t>Patch models/Attendance.js.</t>
+          <t>npm run test:attendance-leave-request-id</t>
         </is>
       </c>
     </row>
@@ -2052,7 +2052,7 @@
       </c>
       <c r="F26" s="4" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Verified</t>
         </is>
       </c>
       <c r="G26" s="4" t="inlineStr">
@@ -2072,7 +2072,7 @@
       </c>
       <c r="J26" s="4" t="inlineStr">
         <is>
-          <t>Call on every approval (and after swap creates approved rows).</t>
+          <t>npm run test:sync-attendance-for-leave</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add leaveRoutes.js leave API route module
</commit_message>
<xml_diff>
--- a/Leave-Payroll-Implementation-Tracker.xlsx
+++ b/Leave-Payroll-Implementation-Tracker.xlsx
@@ -2104,7 +2104,7 @@
       </c>
       <c r="F27" s="4" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Verified</t>
         </is>
       </c>
       <c r="G27" s="4" t="inlineStr">
@@ -2122,7 +2122,11 @@
           <t>Leave Stage 6</t>
         </is>
       </c>
-      <c r="J27" s="4" t="inlineStr"/>
+      <c r="J27" s="4" t="inlineStr">
+        <is>
+          <t>npm run test:approve-leave-attendance</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -2168,7 +2172,7 @@
       </c>
       <c r="F29" s="4" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="G29" s="4" t="inlineStr">
@@ -2186,7 +2190,11 @@
           <t>Leave Stage 7</t>
         </is>
       </c>
-      <c r="J29" s="4" t="inlineStr"/>
+      <c r="J29" s="4" t="inlineStr">
+        <is>
+          <t>backend/routes/leaveRoutes.js — auth middleware; endpoints in rows 31–35.</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="4" t="inlineStr">

</xml_diff>

<commit_message>
Mount leaveRoutes at /api/leave in preciousRoutes
</commit_message>
<xml_diff>
--- a/Leave-Payroll-Implementation-Tracker.xlsx
+++ b/Leave-Payroll-Implementation-Tracker.xlsx
@@ -2224,7 +2224,7 @@
       </c>
       <c r="F30" s="4" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="G30" s="4" t="inlineStr">
@@ -2242,7 +2242,11 @@
           <t>Leave Stage 7</t>
         </is>
       </c>
-      <c r="J30" s="4" t="inlineStr"/>
+      <c r="J30" s="4" t="inlineStr">
+        <is>
+          <t>Mounted at /api/leave via preciousRoutes.js</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="4" t="inlineStr">

</xml_diff>

<commit_message>
Add POST /api/leave/request with clash and is_paid checks
</commit_message>
<xml_diff>
--- a/Leave-Payroll-Implementation-Tracker.xlsx
+++ b/Leave-Payroll-Implementation-Tracker.xlsx
@@ -2276,7 +2276,7 @@
       </c>
       <c r="F31" s="4" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Verified</t>
         </is>
       </c>
       <c r="G31" s="4" t="inlineStr">
@@ -2294,7 +2294,11 @@
           <t>Leave Stage 7</t>
         </is>
       </c>
-      <c r="J31" s="4" t="inlineStr"/>
+      <c r="J31" s="4" t="inlineStr">
+        <is>
+          <t>npm run test:leave-request-api</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="4" t="inlineStr">

</xml_diff>

<commit_message>
Add POST /api/leave/:id/approve with attendance sync
</commit_message>
<xml_diff>
--- a/Leave-Payroll-Implementation-Tracker.xlsx
+++ b/Leave-Payroll-Implementation-Tracker.xlsx
@@ -2328,7 +2328,7 @@
       </c>
       <c r="F32" s="4" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Verified</t>
         </is>
       </c>
       <c r="G32" s="4" t="inlineStr">
@@ -2346,7 +2346,11 @@
           <t>Leave Stage 7</t>
         </is>
       </c>
-      <c r="J32" s="4" t="inlineStr"/>
+      <c r="J32" s="4" t="inlineStr">
+        <is>
+          <t>npm run test:leave-approve-api</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="4" t="inlineStr">

</xml_diff>

<commit_message>
Add full leave API happy path integration test
</commit_message>
<xml_diff>
--- a/Leave-Payroll-Implementation-Tracker.xlsx
+++ b/Leave-Payroll-Implementation-Tracker.xlsx
@@ -2380,7 +2380,7 @@
       </c>
       <c r="F33" s="4" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Verified</t>
         </is>
       </c>
       <c r="G33" s="4" t="inlineStr">
@@ -2398,7 +2398,11 @@
           <t>Leave Stage 7</t>
         </is>
       </c>
-      <c r="J33" s="4" t="inlineStr"/>
+      <c r="J33" s="4" t="inlineStr">
+        <is>
+          <t>npm run test:leave-reject-api</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="4" t="inlineStr">
@@ -2428,7 +2432,7 @@
       </c>
       <c r="F34" s="4" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Verified</t>
         </is>
       </c>
       <c r="G34" s="4" t="inlineStr">
@@ -2446,7 +2450,11 @@
           <t>Leave Stage 7</t>
         </is>
       </c>
-      <c r="J34" s="4" t="inlineStr"/>
+      <c r="J34" s="4" t="inlineStr">
+        <is>
+          <t>npm run test:leave-swap-api</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="4" t="inlineStr">
@@ -2476,7 +2484,7 @@
       </c>
       <c r="F35" s="4" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Verified</t>
         </is>
       </c>
       <c r="G35" s="4" t="inlineStr">
@@ -2494,7 +2502,11 @@
           <t>Leave Stage 7</t>
         </is>
       </c>
-      <c r="J35" s="4" t="inlineStr"/>
+      <c r="J35" s="4" t="inlineStr">
+        <is>
+          <t>npm run test:leave-list-api</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="4" t="inlineStr">
@@ -2524,7 +2536,7 @@
       </c>
       <c r="F36" s="4" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Verified</t>
         </is>
       </c>
       <c r="G36" s="4" t="inlineStr">
@@ -2542,7 +2554,11 @@
           <t>Leave Stage 7</t>
         </is>
       </c>
-      <c r="J36" s="4" t="inlineStr"/>
+      <c r="J36" s="4" t="inlineStr">
+        <is>
+          <t>npm run test:leave-happy-path</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>